<commit_message>
Módulo 4: paleta azul oscuro (en lugar de ciruela) en la presentación y la plantilla Dashboard; 2024 en naranja en los gráficos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Modulo4-Base-Dashboard.xlsx
+++ b/Modulo4-Base-Dashboard.xlsx
@@ -1267,30 +1267,30 @@
     </font>
     <font>
       <i/>
-      <color rgb="FF6B6070"/>
+      <color rgb="FF5C6677"/>
       <sz val="10"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF4A2448"/>
+      <color rgb="FF13315C"/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <color rgb="FF6B6070"/>
+      <color rgb="FF5C6677"/>
       <sz val="12"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF4A2448"/>
+      <color rgb="FF13315C"/>
       <sz val="28"/>
       <name val="Calibri"/>
     </font>
     <font>
       <i/>
-      <color rgb="FF6B6070"/>
+      <color rgb="FF5C6677"/>
       <sz val="9"/>
       <name val="Calibri"/>
     </font>
@@ -1315,7 +1315,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF4A2448"/>
+        <fgColor rgb="FF13315C"/>
       </patternFill>
     </fill>
     <fill>
@@ -1325,7 +1325,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF3EEF6"/>
+        <fgColor rgb="FFEEF2F8"/>
       </patternFill>
     </fill>
     <fill>
@@ -1345,24 +1345,24 @@
     <border>
       <left/>
       <right style="thin">
-        <color rgb="FFCFC6D6"/>
+        <color rgb="FFC9D1DD"/>
       </right>
       <top/>
       <bottom style="thin">
-        <color rgb="FFCFC6D6"/>
+        <color rgb="FFC9D1DD"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right style="thin">
-        <color rgb="FFCFC6D6"/>
+        <color rgb="FFC9D1DD"/>
       </right>
       <top style="thin">
-        <color rgb="FFCFC6D6"/>
+        <color rgb="FFC9D1DD"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFCFC6D6"/>
+        <color rgb="FFC9D1DD"/>
       </bottom>
       <diagonal/>
     </border>

</xml_diff>

<commit_message>
Módulo 4 alineado con Excel para la web: segmentación por Analizar tabla dinámica › Segmentación, conexiones por Configuración de segmentación › Conexiones de tabla dinámica, gráficos con Insertar › Línea/Columna, y todo construido en la hoja Dashboard (tablas dinámicas en la columna T, sin cortar y pegar gráficos)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Modulo4-Base-Dashboard.xlsx
+++ b/Modulo4-Base-Dashboard.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1826" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1831" uniqueCount="413">
   <si>
     <t>ID Servicio</t>
   </si>
@@ -1197,6 +1197,12 @@
   </si>
   <si>
     <t>Fuente: tabla tblServicios (360 servicios, enero 2024 – diciembre 2025). Usa las segmentaciones de la derecha para filtrar todo el tablero.</t>
+  </si>
+  <si>
+    <t>Motor del tablero · tablas dinámicas (no borrar)</t>
+  </si>
+  <si>
+    <t>TD_KPI · crea la tabla dinámica en T5 (solo Valores)</t>
   </si>
   <si>
     <t>Servicios atendidos</t>
@@ -1215,7 +1221,10 @@
     <t/>
   </si>
   <si>
-    <t>↑ En cada tarjeta escribe = y haz clic en el número de TD_KPI.</t>
+    <t>↑ En cada tarjeta escribe = y haz clic en el número de TD_KPI (T6, U6 o V6).</t>
+  </si>
+  <si>
+    <t>TD_Mes · crea la tabla dinámica en T10</t>
   </si>
   <si>
     <t xml:space="preserve">Gráfico 1 · Servicios por mes, 2024 frente a 2025 (Líneas)
@@ -1228,6 +1237,12 @@
   <si>
     <t xml:space="preserve">Gráfico 3 · Servicios por provincia (Columnas)
 Pega aquí el gráfico de TD_Prov</t>
+  </si>
+  <si>
+    <t>TD_ARS · crea la tabla dinámica en T29</t>
+  </si>
+  <si>
+    <t>TD_Prov · crea la tabla dinámica en T38</t>
   </si>
   <si>
     <t>Conclusiones para la dirección (dato + comparación + recomendación)</t>
@@ -1251,7 +1266,7 @@
     <numFmt numFmtId="165" formatCode="&quot;RD$&quot; #,##0"/>
     <numFmt numFmtId="166" formatCode="&quot;RD$&quot; #,##0.00"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -1268,6 +1283,18 @@
     <font>
       <i/>
       <color rgb="FF5C6677"/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF13315C"/>
       <sz val="10"/>
       <name val="Calibri"/>
     </font>
@@ -1325,12 +1352,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEEF2F8"/>
+        <fgColor rgb="FFE8F1FB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE8F1FB"/>
+        <fgColor rgb="FFEEF2F8"/>
       </patternFill>
     </fill>
   </fills>
@@ -1370,7 +1397,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1380,31 +1407,37 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -12991,13 +13024,15 @@
   <sheetPr>
     <tabColor rgb="FF2F86D6"/>
   </sheetPr>
-  <dimension ref="B1:Q48"/>
+  <dimension ref="B1:W48"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="13" width="11" customWidth="1"/>
     <col min="14" max="14" width="3" customWidth="1"/>
     <col min="15" max="17" width="12" customWidth="1"/>
+    <col min="18" max="19" width="3" customWidth="1"/>
+    <col min="20" max="23" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="2:17" x14ac:dyDescent="0.25">
@@ -13038,7 +13073,7 @@
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
     </row>
-    <row r="3" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
         <v>394</v>
       </c>
@@ -13057,752 +13092,786 @@
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
+      <c r="T3" s="5" t="s">
+        <v>395</v>
+      </c>
+      <c r="U3" s="5"/>
+      <c r="V3" s="5"/>
+      <c r="W3" s="5"/>
+    </row>
+    <row r="4" spans="20:23" x14ac:dyDescent="0.25">
+      <c r="T4" s="6" t="s">
+        <v>396</v>
+      </c>
+      <c r="U4" s="6"/>
+      <c r="V4" s="6"/>
+      <c r="W4" s="6"/>
     </row>
     <row r="5" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B5" s="5" t="s">
-        <v>395</v>
-      </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5" t="s">
-        <v>396</v>
-      </c>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5" t="s">
+      <c r="B5" s="7" t="s">
         <v>397</v>
       </c>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
-      <c r="O5" s="6" t="s">
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7" t="s">
         <v>398</v>
       </c>
-      <c r="P5" s="6"/>
-      <c r="Q5" s="6"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7" t="s">
+        <v>399</v>
+      </c>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="O5" s="8" t="s">
+        <v>400</v>
+      </c>
+      <c r="P5" s="8"/>
+      <c r="Q5" s="8"/>
     </row>
     <row r="6" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B6" s="7" t="s">
-        <v>399</v>
-      </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="8" t="s">
-        <v>399</v>
-      </c>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="9" t="s">
-        <v>399</v>
-      </c>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="9"/>
-      <c r="O6" s="6"/>
-      <c r="P6" s="6"/>
-      <c r="Q6" s="6"/>
+      <c r="B6" s="9" t="s">
+        <v>401</v>
+      </c>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="10" t="s">
+        <v>401</v>
+      </c>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="11" t="s">
+        <v>401</v>
+      </c>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11"/>
+      <c r="M6" s="11"/>
+      <c r="O6" s="8"/>
+      <c r="P6" s="8"/>
+      <c r="Q6" s="8"/>
     </row>
     <row r="7" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="9"/>
-      <c r="O7" s="6"/>
-      <c r="P7" s="6"/>
-      <c r="Q7" s="6"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10"/>
+      <c r="J7" s="11"/>
+      <c r="K7" s="11"/>
+      <c r="L7" s="11"/>
+      <c r="M7" s="11"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="8"/>
     </row>
     <row r="8" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="9"/>
-      <c r="O8" s="6"/>
-      <c r="P8" s="6"/>
-      <c r="Q8" s="6"/>
-    </row>
-    <row r="9" ht="16" customHeight="1" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B9" s="10" t="s">
-        <v>400</v>
-      </c>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
-      <c r="K9" s="10"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="10"/>
-      <c r="O9" s="6"/>
-      <c r="P9" s="6"/>
-      <c r="Q9" s="6"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="11"/>
+      <c r="K8" s="11"/>
+      <c r="L8" s="11"/>
+      <c r="M8" s="11"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
+    </row>
+    <row r="9" ht="16" customHeight="1" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B9" s="12" t="s">
+        <v>402</v>
+      </c>
+      <c r="C9" s="12"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="12"/>
+      <c r="L9" s="12"/>
+      <c r="M9" s="12"/>
+      <c r="O9" s="8"/>
+      <c r="P9" s="8"/>
+      <c r="Q9" s="8"/>
+      <c r="T9" s="6" t="s">
+        <v>403</v>
+      </c>
+      <c r="U9" s="6"/>
+      <c r="V9" s="6"/>
+      <c r="W9" s="6"/>
     </row>
     <row r="10" spans="15:17" x14ac:dyDescent="0.25">
-      <c r="O10" s="6"/>
-      <c r="P10" s="6"/>
-      <c r="Q10" s="6"/>
+      <c r="O10" s="8"/>
+      <c r="P10" s="8"/>
+      <c r="Q10" s="8"/>
     </row>
     <row r="11" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B11" s="11" t="s">
-        <v>401</v>
-      </c>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="11"/>
-      <c r="L11" s="11"/>
-      <c r="M11" s="11"/>
-      <c r="O11" s="6"/>
-      <c r="P11" s="6"/>
-      <c r="Q11" s="6"/>
+      <c r="B11" s="13" t="s">
+        <v>404</v>
+      </c>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="13"/>
+      <c r="J11" s="13"/>
+      <c r="K11" s="13"/>
+      <c r="L11" s="13"/>
+      <c r="M11" s="13"/>
+      <c r="O11" s="8"/>
+      <c r="P11" s="8"/>
+      <c r="Q11" s="8"/>
     </row>
     <row r="12" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="11"/>
-      <c r="I12" s="11"/>
-      <c r="J12" s="11"/>
-      <c r="K12" s="11"/>
-      <c r="L12" s="11"/>
-      <c r="M12" s="11"/>
-      <c r="O12" s="6"/>
-      <c r="P12" s="6"/>
-      <c r="Q12" s="6"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="13"/>
+      <c r="J12" s="13"/>
+      <c r="K12" s="13"/>
+      <c r="L12" s="13"/>
+      <c r="M12" s="13"/>
+      <c r="O12" s="8"/>
+      <c r="P12" s="8"/>
+      <c r="Q12" s="8"/>
     </row>
     <row r="13" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
-      <c r="I13" s="11"/>
-      <c r="J13" s="11"/>
-      <c r="K13" s="11"/>
-      <c r="L13" s="11"/>
-      <c r="M13" s="11"/>
-      <c r="O13" s="6"/>
-      <c r="P13" s="6"/>
-      <c r="Q13" s="6"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="13"/>
+      <c r="J13" s="13"/>
+      <c r="K13" s="13"/>
+      <c r="L13" s="13"/>
+      <c r="M13" s="13"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="8"/>
+      <c r="Q13" s="8"/>
     </row>
     <row r="14" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="11"/>
-      <c r="I14" s="11"/>
-      <c r="J14" s="11"/>
-      <c r="K14" s="11"/>
-      <c r="L14" s="11"/>
-      <c r="M14" s="11"/>
-      <c r="O14" s="6"/>
-      <c r="P14" s="6"/>
-      <c r="Q14" s="6"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+      <c r="H14" s="13"/>
+      <c r="I14" s="13"/>
+      <c r="J14" s="13"/>
+      <c r="K14" s="13"/>
+      <c r="L14" s="13"/>
+      <c r="M14" s="13"/>
+      <c r="O14" s="8"/>
+      <c r="P14" s="8"/>
+      <c r="Q14" s="8"/>
     </row>
     <row r="15" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="11"/>
-      <c r="J15" s="11"/>
-      <c r="K15" s="11"/>
-      <c r="L15" s="11"/>
-      <c r="M15" s="11"/>
-      <c r="O15" s="6"/>
-      <c r="P15" s="6"/>
-      <c r="Q15" s="6"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="13"/>
+      <c r="J15" s="13"/>
+      <c r="K15" s="13"/>
+      <c r="L15" s="13"/>
+      <c r="M15" s="13"/>
+      <c r="O15" s="8"/>
+      <c r="P15" s="8"/>
+      <c r="Q15" s="8"/>
     </row>
     <row r="16" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="11"/>
-      <c r="J16" s="11"/>
-      <c r="K16" s="11"/>
-      <c r="L16" s="11"/>
-      <c r="M16" s="11"/>
-      <c r="O16" s="6"/>
-      <c r="P16" s="6"/>
-      <c r="Q16" s="6"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="13"/>
+      <c r="I16" s="13"/>
+      <c r="J16" s="13"/>
+      <c r="K16" s="13"/>
+      <c r="L16" s="13"/>
+      <c r="M16" s="13"/>
+      <c r="O16" s="8"/>
+      <c r="P16" s="8"/>
+      <c r="Q16" s="8"/>
     </row>
     <row r="17" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="11"/>
-      <c r="J17" s="11"/>
-      <c r="K17" s="11"/>
-      <c r="L17" s="11"/>
-      <c r="M17" s="11"/>
-      <c r="O17" s="6"/>
-      <c r="P17" s="6"/>
-      <c r="Q17" s="6"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="13"/>
+      <c r="I17" s="13"/>
+      <c r="J17" s="13"/>
+      <c r="K17" s="13"/>
+      <c r="L17" s="13"/>
+      <c r="M17" s="13"/>
+      <c r="O17" s="8"/>
+      <c r="P17" s="8"/>
+      <c r="Q17" s="8"/>
     </row>
     <row r="18" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="11"/>
-      <c r="J18" s="11"/>
-      <c r="K18" s="11"/>
-      <c r="L18" s="11"/>
-      <c r="M18" s="11"/>
-      <c r="O18" s="6"/>
-      <c r="P18" s="6"/>
-      <c r="Q18" s="6"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="13"/>
+      <c r="I18" s="13"/>
+      <c r="J18" s="13"/>
+      <c r="K18" s="13"/>
+      <c r="L18" s="13"/>
+      <c r="M18" s="13"/>
+      <c r="O18" s="8"/>
+      <c r="P18" s="8"/>
+      <c r="Q18" s="8"/>
     </row>
     <row r="19" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B19" s="11"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="11"/>
-      <c r="J19" s="11"/>
-      <c r="K19" s="11"/>
-      <c r="L19" s="11"/>
-      <c r="M19" s="11"/>
-      <c r="O19" s="6"/>
-      <c r="P19" s="6"/>
-      <c r="Q19" s="6"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="13"/>
+      <c r="I19" s="13"/>
+      <c r="J19" s="13"/>
+      <c r="K19" s="13"/>
+      <c r="L19" s="13"/>
+      <c r="M19" s="13"/>
+      <c r="O19" s="8"/>
+      <c r="P19" s="8"/>
+      <c r="Q19" s="8"/>
     </row>
     <row r="20" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B20" s="11"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="11"/>
-      <c r="J20" s="11"/>
-      <c r="K20" s="11"/>
-      <c r="L20" s="11"/>
-      <c r="M20" s="11"/>
-      <c r="O20" s="6"/>
-      <c r="P20" s="6"/>
-      <c r="Q20" s="6"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="13"/>
+      <c r="I20" s="13"/>
+      <c r="J20" s="13"/>
+      <c r="K20" s="13"/>
+      <c r="L20" s="13"/>
+      <c r="M20" s="13"/>
+      <c r="O20" s="8"/>
+      <c r="P20" s="8"/>
+      <c r="Q20" s="8"/>
     </row>
     <row r="21" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="11"/>
-      <c r="L21" s="11"/>
-      <c r="M21" s="11"/>
-      <c r="O21" s="6"/>
-      <c r="P21" s="6"/>
-      <c r="Q21" s="6"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="13"/>
+      <c r="H21" s="13"/>
+      <c r="I21" s="13"/>
+      <c r="J21" s="13"/>
+      <c r="K21" s="13"/>
+      <c r="L21" s="13"/>
+      <c r="M21" s="13"/>
+      <c r="O21" s="8"/>
+      <c r="P21" s="8"/>
+      <c r="Q21" s="8"/>
     </row>
     <row r="22" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B22" s="11"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="11"/>
-      <c r="J22" s="11"/>
-      <c r="K22" s="11"/>
-      <c r="L22" s="11"/>
-      <c r="M22" s="11"/>
-      <c r="O22" s="6"/>
-      <c r="P22" s="6"/>
-      <c r="Q22" s="6"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="13"/>
+      <c r="H22" s="13"/>
+      <c r="I22" s="13"/>
+      <c r="J22" s="13"/>
+      <c r="K22" s="13"/>
+      <c r="L22" s="13"/>
+      <c r="M22" s="13"/>
+      <c r="O22" s="8"/>
+      <c r="P22" s="8"/>
+      <c r="Q22" s="8"/>
     </row>
     <row r="23" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B23" s="11"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="11"/>
-      <c r="J23" s="11"/>
-      <c r="K23" s="11"/>
-      <c r="L23" s="11"/>
-      <c r="M23" s="11"/>
-      <c r="O23" s="6"/>
-      <c r="P23" s="6"/>
-      <c r="Q23" s="6"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+      <c r="G23" s="13"/>
+      <c r="H23" s="13"/>
+      <c r="I23" s="13"/>
+      <c r="J23" s="13"/>
+      <c r="K23" s="13"/>
+      <c r="L23" s="13"/>
+      <c r="M23" s="13"/>
+      <c r="O23" s="8"/>
+      <c r="P23" s="8"/>
+      <c r="Q23" s="8"/>
     </row>
     <row r="24" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B24" s="11"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="11"/>
-      <c r="H24" s="11"/>
-      <c r="I24" s="11"/>
-      <c r="J24" s="11"/>
-      <c r="K24" s="11"/>
-      <c r="L24" s="11"/>
-      <c r="M24" s="11"/>
-      <c r="O24" s="6"/>
-      <c r="P24" s="6"/>
-      <c r="Q24" s="6"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="13"/>
+      <c r="G24" s="13"/>
+      <c r="H24" s="13"/>
+      <c r="I24" s="13"/>
+      <c r="J24" s="13"/>
+      <c r="K24" s="13"/>
+      <c r="L24" s="13"/>
+      <c r="M24" s="13"/>
+      <c r="O24" s="8"/>
+      <c r="P24" s="8"/>
+      <c r="Q24" s="8"/>
     </row>
     <row r="25" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B25" s="11"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="11"/>
-      <c r="J25" s="11"/>
-      <c r="K25" s="11"/>
-      <c r="L25" s="11"/>
-      <c r="M25" s="11"/>
-      <c r="O25" s="6"/>
-      <c r="P25" s="6"/>
-      <c r="Q25" s="6"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="13"/>
+      <c r="G25" s="13"/>
+      <c r="H25" s="13"/>
+      <c r="I25" s="13"/>
+      <c r="J25" s="13"/>
+      <c r="K25" s="13"/>
+      <c r="L25" s="13"/>
+      <c r="M25" s="13"/>
+      <c r="O25" s="8"/>
+      <c r="P25" s="8"/>
+      <c r="Q25" s="8"/>
     </row>
     <row r="26" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B26" s="11"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="11"/>
-      <c r="H26" s="11"/>
-      <c r="I26" s="11"/>
-      <c r="J26" s="11"/>
-      <c r="K26" s="11"/>
-      <c r="L26" s="11"/>
-      <c r="M26" s="11"/>
-      <c r="O26" s="6"/>
-      <c r="P26" s="6"/>
-      <c r="Q26" s="6"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="13"/>
+      <c r="H26" s="13"/>
+      <c r="I26" s="13"/>
+      <c r="J26" s="13"/>
+      <c r="K26" s="13"/>
+      <c r="L26" s="13"/>
+      <c r="M26" s="13"/>
+      <c r="O26" s="8"/>
+      <c r="P26" s="8"/>
+      <c r="Q26" s="8"/>
     </row>
     <row r="27" spans="15:17" x14ac:dyDescent="0.25">
-      <c r="O27" s="6"/>
-      <c r="P27" s="6"/>
-      <c r="Q27" s="6"/>
-    </row>
-    <row r="28" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B28" s="11" t="s">
-        <v>402</v>
-      </c>
-      <c r="C28" s="11"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="11"/>
-      <c r="G28" s="11"/>
-      <c r="H28" s="11" t="s">
-        <v>403</v>
-      </c>
-      <c r="I28" s="11"/>
-      <c r="J28" s="11"/>
-      <c r="K28" s="11"/>
-      <c r="L28" s="11"/>
-      <c r="M28" s="11"/>
-      <c r="O28" s="6"/>
-      <c r="P28" s="6"/>
-      <c r="Q28" s="6"/>
+      <c r="O27" s="8"/>
+      <c r="P27" s="8"/>
+      <c r="Q27" s="8"/>
+    </row>
+    <row r="28" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B28" s="13" t="s">
+        <v>405</v>
+      </c>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="13"/>
+      <c r="G28" s="13"/>
+      <c r="H28" s="13" t="s">
+        <v>406</v>
+      </c>
+      <c r="I28" s="13"/>
+      <c r="J28" s="13"/>
+      <c r="K28" s="13"/>
+      <c r="L28" s="13"/>
+      <c r="M28" s="13"/>
+      <c r="O28" s="8"/>
+      <c r="P28" s="8"/>
+      <c r="Q28" s="8"/>
+      <c r="T28" s="6" t="s">
+        <v>407</v>
+      </c>
+      <c r="U28" s="6"/>
+      <c r="V28" s="6"/>
+      <c r="W28" s="6"/>
     </row>
     <row r="29" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B29" s="11"/>
-      <c r="C29" s="11"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="11"/>
-      <c r="F29" s="11"/>
-      <c r="G29" s="11"/>
-      <c r="H29" s="11"/>
-      <c r="I29" s="11"/>
-      <c r="J29" s="11"/>
-      <c r="K29" s="11"/>
-      <c r="L29" s="11"/>
-      <c r="M29" s="11"/>
-      <c r="O29" s="6"/>
-      <c r="P29" s="6"/>
-      <c r="Q29" s="6"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="13"/>
+      <c r="G29" s="13"/>
+      <c r="H29" s="13"/>
+      <c r="I29" s="13"/>
+      <c r="J29" s="13"/>
+      <c r="K29" s="13"/>
+      <c r="L29" s="13"/>
+      <c r="M29" s="13"/>
+      <c r="O29" s="8"/>
+      <c r="P29" s="8"/>
+      <c r="Q29" s="8"/>
     </row>
     <row r="30" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B30" s="11"/>
-      <c r="C30" s="11"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="11"/>
-      <c r="G30" s="11"/>
-      <c r="H30" s="11"/>
-      <c r="I30" s="11"/>
-      <c r="J30" s="11"/>
-      <c r="K30" s="11"/>
-      <c r="L30" s="11"/>
-      <c r="M30" s="11"/>
-      <c r="O30" s="6"/>
-      <c r="P30" s="6"/>
-      <c r="Q30" s="6"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="13"/>
+      <c r="F30" s="13"/>
+      <c r="G30" s="13"/>
+      <c r="H30" s="13"/>
+      <c r="I30" s="13"/>
+      <c r="J30" s="13"/>
+      <c r="K30" s="13"/>
+      <c r="L30" s="13"/>
+      <c r="M30" s="13"/>
+      <c r="O30" s="8"/>
+      <c r="P30" s="8"/>
+      <c r="Q30" s="8"/>
     </row>
     <row r="31" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B31" s="11"/>
-      <c r="C31" s="11"/>
-      <c r="D31" s="11"/>
-      <c r="E31" s="11"/>
-      <c r="F31" s="11"/>
-      <c r="G31" s="11"/>
-      <c r="H31" s="11"/>
-      <c r="I31" s="11"/>
-      <c r="J31" s="11"/>
-      <c r="K31" s="11"/>
-      <c r="L31" s="11"/>
-      <c r="M31" s="11"/>
-      <c r="O31" s="6"/>
-      <c r="P31" s="6"/>
-      <c r="Q31" s="6"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
+      <c r="F31" s="13"/>
+      <c r="G31" s="13"/>
+      <c r="H31" s="13"/>
+      <c r="I31" s="13"/>
+      <c r="J31" s="13"/>
+      <c r="K31" s="13"/>
+      <c r="L31" s="13"/>
+      <c r="M31" s="13"/>
+      <c r="O31" s="8"/>
+      <c r="P31" s="8"/>
+      <c r="Q31" s="8"/>
     </row>
     <row r="32" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B32" s="11"/>
-      <c r="C32" s="11"/>
-      <c r="D32" s="11"/>
-      <c r="E32" s="11"/>
-      <c r="F32" s="11"/>
-      <c r="G32" s="11"/>
-      <c r="H32" s="11"/>
-      <c r="I32" s="11"/>
-      <c r="J32" s="11"/>
-      <c r="K32" s="11"/>
-      <c r="L32" s="11"/>
-      <c r="M32" s="11"/>
-      <c r="O32" s="6"/>
-      <c r="P32" s="6"/>
-      <c r="Q32" s="6"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="13"/>
+      <c r="F32" s="13"/>
+      <c r="G32" s="13"/>
+      <c r="H32" s="13"/>
+      <c r="I32" s="13"/>
+      <c r="J32" s="13"/>
+      <c r="K32" s="13"/>
+      <c r="L32" s="13"/>
+      <c r="M32" s="13"/>
+      <c r="O32" s="8"/>
+      <c r="P32" s="8"/>
+      <c r="Q32" s="8"/>
     </row>
     <row r="33" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B33" s="11"/>
-      <c r="C33" s="11"/>
-      <c r="D33" s="11"/>
-      <c r="E33" s="11"/>
-      <c r="F33" s="11"/>
-      <c r="G33" s="11"/>
-      <c r="H33" s="11"/>
-      <c r="I33" s="11"/>
-      <c r="J33" s="11"/>
-      <c r="K33" s="11"/>
-      <c r="L33" s="11"/>
-      <c r="M33" s="11"/>
-      <c r="O33" s="6"/>
-      <c r="P33" s="6"/>
-      <c r="Q33" s="6"/>
+      <c r="B33" s="13"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="13"/>
+      <c r="F33" s="13"/>
+      <c r="G33" s="13"/>
+      <c r="H33" s="13"/>
+      <c r="I33" s="13"/>
+      <c r="J33" s="13"/>
+      <c r="K33" s="13"/>
+      <c r="L33" s="13"/>
+      <c r="M33" s="13"/>
+      <c r="O33" s="8"/>
+      <c r="P33" s="8"/>
+      <c r="Q33" s="8"/>
     </row>
     <row r="34" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B34" s="11"/>
-      <c r="C34" s="11"/>
-      <c r="D34" s="11"/>
-      <c r="E34" s="11"/>
-      <c r="F34" s="11"/>
-      <c r="G34" s="11"/>
-      <c r="H34" s="11"/>
-      <c r="I34" s="11"/>
-      <c r="J34" s="11"/>
-      <c r="K34" s="11"/>
-      <c r="L34" s="11"/>
-      <c r="M34" s="11"/>
-      <c r="O34" s="6"/>
-      <c r="P34" s="6"/>
-      <c r="Q34" s="6"/>
+      <c r="B34" s="13"/>
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="13"/>
+      <c r="F34" s="13"/>
+      <c r="G34" s="13"/>
+      <c r="H34" s="13"/>
+      <c r="I34" s="13"/>
+      <c r="J34" s="13"/>
+      <c r="K34" s="13"/>
+      <c r="L34" s="13"/>
+      <c r="M34" s="13"/>
+      <c r="O34" s="8"/>
+      <c r="P34" s="8"/>
+      <c r="Q34" s="8"/>
     </row>
     <row r="35" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B35" s="11"/>
-      <c r="C35" s="11"/>
-      <c r="D35" s="11"/>
-      <c r="E35" s="11"/>
-      <c r="F35" s="11"/>
-      <c r="G35" s="11"/>
-      <c r="H35" s="11"/>
-      <c r="I35" s="11"/>
-      <c r="J35" s="11"/>
-      <c r="K35" s="11"/>
-      <c r="L35" s="11"/>
-      <c r="M35" s="11"/>
-      <c r="O35" s="6"/>
-      <c r="P35" s="6"/>
-      <c r="Q35" s="6"/>
+      <c r="B35" s="13"/>
+      <c r="C35" s="13"/>
+      <c r="D35" s="13"/>
+      <c r="E35" s="13"/>
+      <c r="F35" s="13"/>
+      <c r="G35" s="13"/>
+      <c r="H35" s="13"/>
+      <c r="I35" s="13"/>
+      <c r="J35" s="13"/>
+      <c r="K35" s="13"/>
+      <c r="L35" s="13"/>
+      <c r="M35" s="13"/>
+      <c r="O35" s="8"/>
+      <c r="P35" s="8"/>
+      <c r="Q35" s="8"/>
     </row>
     <row r="36" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B36" s="11"/>
-      <c r="C36" s="11"/>
-      <c r="D36" s="11"/>
-      <c r="E36" s="11"/>
-      <c r="F36" s="11"/>
-      <c r="G36" s="11"/>
-      <c r="H36" s="11"/>
-      <c r="I36" s="11"/>
-      <c r="J36" s="11"/>
-      <c r="K36" s="11"/>
-      <c r="L36" s="11"/>
-      <c r="M36" s="11"/>
-      <c r="O36" s="6"/>
-      <c r="P36" s="6"/>
-      <c r="Q36" s="6"/>
-    </row>
-    <row r="37" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B37" s="11"/>
-      <c r="C37" s="11"/>
-      <c r="D37" s="11"/>
-      <c r="E37" s="11"/>
-      <c r="F37" s="11"/>
-      <c r="G37" s="11"/>
-      <c r="H37" s="11"/>
-      <c r="I37" s="11"/>
-      <c r="J37" s="11"/>
-      <c r="K37" s="11"/>
-      <c r="L37" s="11"/>
-      <c r="M37" s="11"/>
-      <c r="O37" s="6"/>
-      <c r="P37" s="6"/>
-      <c r="Q37" s="6"/>
+      <c r="B36" s="13"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="13"/>
+      <c r="F36" s="13"/>
+      <c r="G36" s="13"/>
+      <c r="H36" s="13"/>
+      <c r="I36" s="13"/>
+      <c r="J36" s="13"/>
+      <c r="K36" s="13"/>
+      <c r="L36" s="13"/>
+      <c r="M36" s="13"/>
+      <c r="O36" s="8"/>
+      <c r="P36" s="8"/>
+      <c r="Q36" s="8"/>
+    </row>
+    <row r="37" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B37" s="13"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="13"/>
+      <c r="F37" s="13"/>
+      <c r="G37" s="13"/>
+      <c r="H37" s="13"/>
+      <c r="I37" s="13"/>
+      <c r="J37" s="13"/>
+      <c r="K37" s="13"/>
+      <c r="L37" s="13"/>
+      <c r="M37" s="13"/>
+      <c r="O37" s="8"/>
+      <c r="P37" s="8"/>
+      <c r="Q37" s="8"/>
+      <c r="T37" s="6" t="s">
+        <v>408</v>
+      </c>
+      <c r="U37" s="6"/>
+      <c r="V37" s="6"/>
+      <c r="W37" s="6"/>
     </row>
     <row r="38" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B38" s="11"/>
-      <c r="C38" s="11"/>
-      <c r="D38" s="11"/>
-      <c r="E38" s="11"/>
-      <c r="F38" s="11"/>
-      <c r="G38" s="11"/>
-      <c r="H38" s="11"/>
-      <c r="I38" s="11"/>
-      <c r="J38" s="11"/>
-      <c r="K38" s="11"/>
-      <c r="L38" s="11"/>
-      <c r="M38" s="11"/>
-      <c r="O38" s="6"/>
-      <c r="P38" s="6"/>
-      <c r="Q38" s="6"/>
+      <c r="B38" s="13"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="13"/>
+      <c r="F38" s="13"/>
+      <c r="G38" s="13"/>
+      <c r="H38" s="13"/>
+      <c r="I38" s="13"/>
+      <c r="J38" s="13"/>
+      <c r="K38" s="13"/>
+      <c r="L38" s="13"/>
+      <c r="M38" s="13"/>
+      <c r="O38" s="8"/>
+      <c r="P38" s="8"/>
+      <c r="Q38" s="8"/>
     </row>
     <row r="39" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B39" s="11"/>
-      <c r="C39" s="11"/>
-      <c r="D39" s="11"/>
-      <c r="E39" s="11"/>
-      <c r="F39" s="11"/>
-      <c r="G39" s="11"/>
-      <c r="H39" s="11"/>
-      <c r="I39" s="11"/>
-      <c r="J39" s="11"/>
-      <c r="K39" s="11"/>
-      <c r="L39" s="11"/>
-      <c r="M39" s="11"/>
-      <c r="O39" s="6"/>
-      <c r="P39" s="6"/>
-      <c r="Q39" s="6"/>
+      <c r="B39" s="13"/>
+      <c r="C39" s="13"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="13"/>
+      <c r="F39" s="13"/>
+      <c r="G39" s="13"/>
+      <c r="H39" s="13"/>
+      <c r="I39" s="13"/>
+      <c r="J39" s="13"/>
+      <c r="K39" s="13"/>
+      <c r="L39" s="13"/>
+      <c r="M39" s="13"/>
+      <c r="O39" s="8"/>
+      <c r="P39" s="8"/>
+      <c r="Q39" s="8"/>
     </row>
     <row r="40" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B40" s="11"/>
-      <c r="C40" s="11"/>
-      <c r="D40" s="11"/>
-      <c r="E40" s="11"/>
-      <c r="F40" s="11"/>
-      <c r="G40" s="11"/>
-      <c r="H40" s="11"/>
-      <c r="I40" s="11"/>
-      <c r="J40" s="11"/>
-      <c r="K40" s="11"/>
-      <c r="L40" s="11"/>
-      <c r="M40" s="11"/>
-      <c r="O40" s="6"/>
-      <c r="P40" s="6"/>
-      <c r="Q40" s="6"/>
+      <c r="B40" s="13"/>
+      <c r="C40" s="13"/>
+      <c r="D40" s="13"/>
+      <c r="E40" s="13"/>
+      <c r="F40" s="13"/>
+      <c r="G40" s="13"/>
+      <c r="H40" s="13"/>
+      <c r="I40" s="13"/>
+      <c r="J40" s="13"/>
+      <c r="K40" s="13"/>
+      <c r="L40" s="13"/>
+      <c r="M40" s="13"/>
+      <c r="O40" s="8"/>
+      <c r="P40" s="8"/>
+      <c r="Q40" s="8"/>
     </row>
     <row r="41" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B41" s="11"/>
-      <c r="C41" s="11"/>
-      <c r="D41" s="11"/>
-      <c r="E41" s="11"/>
-      <c r="F41" s="11"/>
-      <c r="G41" s="11"/>
-      <c r="H41" s="11"/>
-      <c r="I41" s="11"/>
-      <c r="J41" s="11"/>
-      <c r="K41" s="11"/>
-      <c r="L41" s="11"/>
-      <c r="M41" s="11"/>
-      <c r="O41" s="6"/>
-      <c r="P41" s="6"/>
-      <c r="Q41" s="6"/>
+      <c r="B41" s="13"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="13"/>
+      <c r="E41" s="13"/>
+      <c r="F41" s="13"/>
+      <c r="G41" s="13"/>
+      <c r="H41" s="13"/>
+      <c r="I41" s="13"/>
+      <c r="J41" s="13"/>
+      <c r="K41" s="13"/>
+      <c r="L41" s="13"/>
+      <c r="M41" s="13"/>
+      <c r="O41" s="8"/>
+      <c r="P41" s="8"/>
+      <c r="Q41" s="8"/>
     </row>
     <row r="42" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B42" s="11"/>
-      <c r="C42" s="11"/>
-      <c r="D42" s="11"/>
-      <c r="E42" s="11"/>
-      <c r="F42" s="11"/>
-      <c r="G42" s="11"/>
-      <c r="H42" s="11"/>
-      <c r="I42" s="11"/>
-      <c r="J42" s="11"/>
-      <c r="K42" s="11"/>
-      <c r="L42" s="11"/>
-      <c r="M42" s="11"/>
-      <c r="O42" s="6"/>
-      <c r="P42" s="6"/>
-      <c r="Q42" s="6"/>
+      <c r="B42" s="13"/>
+      <c r="C42" s="13"/>
+      <c r="D42" s="13"/>
+      <c r="E42" s="13"/>
+      <c r="F42" s="13"/>
+      <c r="G42" s="13"/>
+      <c r="H42" s="13"/>
+      <c r="I42" s="13"/>
+      <c r="J42" s="13"/>
+      <c r="K42" s="13"/>
+      <c r="L42" s="13"/>
+      <c r="M42" s="13"/>
+      <c r="O42" s="8"/>
+      <c r="P42" s="8"/>
+      <c r="Q42" s="8"/>
     </row>
     <row r="43" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B43" s="11"/>
-      <c r="C43" s="11"/>
-      <c r="D43" s="11"/>
-      <c r="E43" s="11"/>
-      <c r="F43" s="11"/>
-      <c r="G43" s="11"/>
-      <c r="H43" s="11"/>
-      <c r="I43" s="11"/>
-      <c r="J43" s="11"/>
-      <c r="K43" s="11"/>
-      <c r="L43" s="11"/>
-      <c r="M43" s="11"/>
-      <c r="O43" s="6"/>
-      <c r="P43" s="6"/>
-      <c r="Q43" s="6"/>
+      <c r="B43" s="13"/>
+      <c r="C43" s="13"/>
+      <c r="D43" s="13"/>
+      <c r="E43" s="13"/>
+      <c r="F43" s="13"/>
+      <c r="G43" s="13"/>
+      <c r="H43" s="13"/>
+      <c r="I43" s="13"/>
+      <c r="J43" s="13"/>
+      <c r="K43" s="13"/>
+      <c r="L43" s="13"/>
+      <c r="M43" s="13"/>
+      <c r="O43" s="8"/>
+      <c r="P43" s="8"/>
+      <c r="Q43" s="8"/>
     </row>
     <row r="45" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B45" s="12" t="s">
-        <v>404</v>
-      </c>
-      <c r="C45" s="12"/>
-      <c r="D45" s="12"/>
-      <c r="E45" s="12"/>
-      <c r="F45" s="12"/>
-      <c r="G45" s="12"/>
-      <c r="H45" s="12"/>
-      <c r="I45" s="12"/>
-      <c r="J45" s="12"/>
-      <c r="K45" s="12"/>
-      <c r="L45" s="12"/>
-      <c r="M45" s="12"/>
-      <c r="N45" s="12"/>
-      <c r="O45" s="12"/>
-      <c r="P45" s="12"/>
-      <c r="Q45" s="12"/>
+      <c r="B45" s="14" t="s">
+        <v>409</v>
+      </c>
+      <c r="C45" s="14"/>
+      <c r="D45" s="14"/>
+      <c r="E45" s="14"/>
+      <c r="F45" s="14"/>
+      <c r="G45" s="14"/>
+      <c r="H45" s="14"/>
+      <c r="I45" s="14"/>
+      <c r="J45" s="14"/>
+      <c r="K45" s="14"/>
+      <c r="L45" s="14"/>
+      <c r="M45" s="14"/>
+      <c r="N45" s="14"/>
+      <c r="O45" s="14"/>
+      <c r="P45" s="14"/>
+      <c r="Q45" s="14"/>
     </row>
     <row r="46" ht="30" customHeight="1" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B46" s="13" t="s">
-        <v>405</v>
-      </c>
-      <c r="C46" s="13"/>
-      <c r="D46" s="13"/>
-      <c r="E46" s="13"/>
-      <c r="F46" s="13"/>
-      <c r="G46" s="13"/>
-      <c r="H46" s="13"/>
-      <c r="I46" s="13"/>
-      <c r="J46" s="13"/>
-      <c r="K46" s="13"/>
-      <c r="L46" s="13"/>
-      <c r="M46" s="13"/>
-      <c r="N46" s="13"/>
-      <c r="O46" s="13"/>
-      <c r="P46" s="13"/>
-      <c r="Q46" s="13"/>
+      <c r="B46" s="15" t="s">
+        <v>410</v>
+      </c>
+      <c r="C46" s="15"/>
+      <c r="D46" s="15"/>
+      <c r="E46" s="15"/>
+      <c r="F46" s="15"/>
+      <c r="G46" s="15"/>
+      <c r="H46" s="15"/>
+      <c r="I46" s="15"/>
+      <c r="J46" s="15"/>
+      <c r="K46" s="15"/>
+      <c r="L46" s="15"/>
+      <c r="M46" s="15"/>
+      <c r="N46" s="15"/>
+      <c r="O46" s="15"/>
+      <c r="P46" s="15"/>
+      <c r="Q46" s="15"/>
     </row>
     <row r="47" ht="30" customHeight="1" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B47" s="13" t="s">
-        <v>406</v>
-      </c>
-      <c r="C47" s="13"/>
-      <c r="D47" s="13"/>
-      <c r="E47" s="13"/>
-      <c r="F47" s="13"/>
-      <c r="G47" s="13"/>
-      <c r="H47" s="13"/>
-      <c r="I47" s="13"/>
-      <c r="J47" s="13"/>
-      <c r="K47" s="13"/>
-      <c r="L47" s="13"/>
-      <c r="M47" s="13"/>
-      <c r="N47" s="13"/>
-      <c r="O47" s="13"/>
-      <c r="P47" s="13"/>
-      <c r="Q47" s="13"/>
+      <c r="B47" s="15" t="s">
+        <v>411</v>
+      </c>
+      <c r="C47" s="15"/>
+      <c r="D47" s="15"/>
+      <c r="E47" s="15"/>
+      <c r="F47" s="15"/>
+      <c r="G47" s="15"/>
+      <c r="H47" s="15"/>
+      <c r="I47" s="15"/>
+      <c r="J47" s="15"/>
+      <c r="K47" s="15"/>
+      <c r="L47" s="15"/>
+      <c r="M47" s="15"/>
+      <c r="N47" s="15"/>
+      <c r="O47" s="15"/>
+      <c r="P47" s="15"/>
+      <c r="Q47" s="15"/>
     </row>
     <row r="48" ht="30" customHeight="1" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B48" s="13" t="s">
-        <v>407</v>
-      </c>
-      <c r="C48" s="13"/>
-      <c r="D48" s="13"/>
-      <c r="E48" s="13"/>
-      <c r="F48" s="13"/>
-      <c r="G48" s="13"/>
-      <c r="H48" s="13"/>
-      <c r="I48" s="13"/>
-      <c r="J48" s="13"/>
-      <c r="K48" s="13"/>
-      <c r="L48" s="13"/>
-      <c r="M48" s="13"/>
-      <c r="N48" s="13"/>
-      <c r="O48" s="13"/>
-      <c r="P48" s="13"/>
-      <c r="Q48" s="13"/>
+      <c r="B48" s="15" t="s">
+        <v>412</v>
+      </c>
+      <c r="C48" s="15"/>
+      <c r="D48" s="15"/>
+      <c r="E48" s="15"/>
+      <c r="F48" s="15"/>
+      <c r="G48" s="15"/>
+      <c r="H48" s="15"/>
+      <c r="I48" s="15"/>
+      <c r="J48" s="15"/>
+      <c r="K48" s="15"/>
+      <c r="L48" s="15"/>
+      <c r="M48" s="15"/>
+      <c r="N48" s="15"/>
+      <c r="O48" s="15"/>
+      <c r="P48" s="15"/>
+      <c r="Q48" s="15"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="22">
     <mergeCell ref="B1:Q2"/>
     <mergeCell ref="B3:Q3"/>
+    <mergeCell ref="T3:W3"/>
+    <mergeCell ref="T4:W4"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="F5:I5"/>
     <mergeCell ref="J5:M5"/>
@@ -13811,9 +13880,12 @@
     <mergeCell ref="F6:I8"/>
     <mergeCell ref="J6:M8"/>
     <mergeCell ref="B9:M9"/>
+    <mergeCell ref="T9:W9"/>
     <mergeCell ref="B11:M26"/>
     <mergeCell ref="B28:G43"/>
     <mergeCell ref="H28:M43"/>
+    <mergeCell ref="T28:W28"/>
+    <mergeCell ref="T37:W37"/>
     <mergeCell ref="B45:Q45"/>
     <mergeCell ref="B46:Q46"/>
     <mergeCell ref="B47:Q47"/>

</xml_diff>

<commit_message>
Módulo 4 remodelado: solo teoría (7 conceptos con ejemplo de ARS + tablero integrador de ARS), abre con la tabla de datos pura; sin simuladores ni prácticas; base Excel sin hoja de plantilla
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Modulo4-Base-Dashboard.xlsx
+++ b/Modulo4-Base-Dashboard.xlsx
@@ -5,14 +5,13 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Servicios" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Dashboard" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1831" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1809" uniqueCount="393">
   <si>
     <t>ID Servicio</t>
   </si>
@@ -1191,82 +1190,16 @@
   </si>
   <si>
     <t>SRV-1360</t>
-  </si>
-  <si>
-    <t>Tablero de servicios de salud · 2024–2025</t>
-  </si>
-  <si>
-    <t>Fuente: tabla tblServicios (360 servicios, enero 2024 – diciembre 2025). Usa las segmentaciones de la derecha para filtrar todo el tablero.</t>
-  </si>
-  <si>
-    <t>Motor del tablero · tablas dinámicas (no borrar)</t>
-  </si>
-  <si>
-    <t>TD_KPI · crea la tabla dinámica en T5 (solo Valores)</t>
-  </si>
-  <si>
-    <t>Servicios atendidos</t>
-  </si>
-  <si>
-    <t>Monto total (RD$)</t>
-  </si>
-  <si>
-    <t>Monto promedio por servicio (RD$)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Segmentaciones
-Pega aquí las segmentaciones de Año y Tipo de Servicio</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>↑ En cada tarjeta escribe = y haz clic en el número de TD_KPI (T6, U6 o V6).</t>
-  </si>
-  <si>
-    <t>TD_Mes · crea la tabla dinámica en T10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gráfico 1 · Servicios por mes, 2024 frente a 2025 (Líneas)
-Pega aquí el gráfico de TD_Mes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gráfico 2 · Monto por ARS (Columnas)
-Pega aquí el gráfico de TD_ARS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gráfico 3 · Servicios por provincia (Columnas)
-Pega aquí el gráfico de TD_Prov</t>
-  </si>
-  <si>
-    <t>TD_ARS · crea la tabla dinámica en T29</t>
-  </si>
-  <si>
-    <t>TD_Prov · crea la tabla dinámica en T38</t>
-  </si>
-  <si>
-    <t>Conclusiones para la dirección (dato + comparación + recomendación)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="3">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="&quot;RD$&quot; #,##0"/>
-    <numFmt numFmtId="166" formatCode="&quot;RD$&quot; #,##0.00"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -1274,94 +1207,16 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="20"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FF5C6677"/>
-      <sz val="10"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF13315C"/>
-      <sz val="10"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF13315C"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <color rgb="FF5C6677"/>
-      <sz val="12"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF13315C"/>
-      <sz val="28"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FF5C6677"/>
-      <sz val="9"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="12"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <color rgb="FF1F1A22"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF13315C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE8F1FB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEEF2F8"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1369,77 +1224,14 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFC9D1DD"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFC9D1DD"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FFC9D1DD"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFC9D1DD"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFC9D1DD"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13017,881 +12809,4 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <tabColor rgb="FF2F86D6"/>
-  </sheetPr>
-  <dimension ref="B1:W48"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="2" customWidth="1"/>
-    <col min="2" max="13" width="11" customWidth="1"/>
-    <col min="14" max="14" width="3" customWidth="1"/>
-    <col min="15" max="17" width="12" customWidth="1"/>
-    <col min="18" max="19" width="3" customWidth="1"/>
-    <col min="20" max="23" width="16" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B1" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
-      <c r="O1" s="3"/>
-      <c r="P1" s="3"/>
-      <c r="Q1" s="3"/>
-    </row>
-    <row r="2" ht="22" customHeight="1" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
-      <c r="P2" s="3"/>
-      <c r="Q2" s="3"/>
-    </row>
-    <row r="3" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B3" s="4" t="s">
-        <v>394</v>
-      </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="4"/>
-      <c r="Q3" s="4"/>
-      <c r="T3" s="5" t="s">
-        <v>395</v>
-      </c>
-      <c r="U3" s="5"/>
-      <c r="V3" s="5"/>
-      <c r="W3" s="5"/>
-    </row>
-    <row r="4" spans="20:23" x14ac:dyDescent="0.25">
-      <c r="T4" s="6" t="s">
-        <v>396</v>
-      </c>
-      <c r="U4" s="6"/>
-      <c r="V4" s="6"/>
-      <c r="W4" s="6"/>
-    </row>
-    <row r="5" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B5" s="7" t="s">
-        <v>397</v>
-      </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7" t="s">
-        <v>398</v>
-      </c>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7" t="s">
-        <v>399</v>
-      </c>
-      <c r="K5" s="7"/>
-      <c r="L5" s="7"/>
-      <c r="M5" s="7"/>
-      <c r="O5" s="8" t="s">
-        <v>400</v>
-      </c>
-      <c r="P5" s="8"/>
-      <c r="Q5" s="8"/>
-    </row>
-    <row r="6" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B6" s="9" t="s">
-        <v>401</v>
-      </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="10" t="s">
-        <v>401</v>
-      </c>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="11" t="s">
-        <v>401</v>
-      </c>
-      <c r="K6" s="11"/>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11"/>
-      <c r="O6" s="8"/>
-      <c r="P6" s="8"/>
-      <c r="Q6" s="8"/>
-    </row>
-    <row r="7" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="11"/>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
-      <c r="O7" s="8"/>
-      <c r="P7" s="8"/>
-      <c r="Q7" s="8"/>
-    </row>
-    <row r="8" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="11"/>
-      <c r="K8" s="11"/>
-      <c r="L8" s="11"/>
-      <c r="M8" s="11"/>
-      <c r="O8" s="8"/>
-      <c r="P8" s="8"/>
-      <c r="Q8" s="8"/>
-    </row>
-    <row r="9" ht="16" customHeight="1" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B9" s="12" t="s">
-        <v>402</v>
-      </c>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="12"/>
-      <c r="L9" s="12"/>
-      <c r="M9" s="12"/>
-      <c r="O9" s="8"/>
-      <c r="P9" s="8"/>
-      <c r="Q9" s="8"/>
-      <c r="T9" s="6" t="s">
-        <v>403</v>
-      </c>
-      <c r="U9" s="6"/>
-      <c r="V9" s="6"/>
-      <c r="W9" s="6"/>
-    </row>
-    <row r="10" spans="15:17" x14ac:dyDescent="0.25">
-      <c r="O10" s="8"/>
-      <c r="P10" s="8"/>
-      <c r="Q10" s="8"/>
-    </row>
-    <row r="11" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B11" s="13" t="s">
-        <v>404</v>
-      </c>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="13"/>
-      <c r="J11" s="13"/>
-      <c r="K11" s="13"/>
-      <c r="L11" s="13"/>
-      <c r="M11" s="13"/>
-      <c r="O11" s="8"/>
-      <c r="P11" s="8"/>
-      <c r="Q11" s="8"/>
-    </row>
-    <row r="12" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="13"/>
-      <c r="J12" s="13"/>
-      <c r="K12" s="13"/>
-      <c r="L12" s="13"/>
-      <c r="M12" s="13"/>
-      <c r="O12" s="8"/>
-      <c r="P12" s="8"/>
-      <c r="Q12" s="8"/>
-    </row>
-    <row r="13" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-      <c r="G13" s="13"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="13"/>
-      <c r="J13" s="13"/>
-      <c r="K13" s="13"/>
-      <c r="L13" s="13"/>
-      <c r="M13" s="13"/>
-      <c r="O13" s="8"/>
-      <c r="P13" s="8"/>
-      <c r="Q13" s="8"/>
-    </row>
-    <row r="14" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="13"/>
-      <c r="I14" s="13"/>
-      <c r="J14" s="13"/>
-      <c r="K14" s="13"/>
-      <c r="L14" s="13"/>
-      <c r="M14" s="13"/>
-      <c r="O14" s="8"/>
-      <c r="P14" s="8"/>
-      <c r="Q14" s="8"/>
-    </row>
-    <row r="15" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B15" s="13"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="13"/>
-      <c r="J15" s="13"/>
-      <c r="K15" s="13"/>
-      <c r="L15" s="13"/>
-      <c r="M15" s="13"/>
-      <c r="O15" s="8"/>
-      <c r="P15" s="8"/>
-      <c r="Q15" s="8"/>
-    </row>
-    <row r="16" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B16" s="13"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="13"/>
-      <c r="J16" s="13"/>
-      <c r="K16" s="13"/>
-      <c r="L16" s="13"/>
-      <c r="M16" s="13"/>
-      <c r="O16" s="8"/>
-      <c r="P16" s="8"/>
-      <c r="Q16" s="8"/>
-    </row>
-    <row r="17" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
-      <c r="I17" s="13"/>
-      <c r="J17" s="13"/>
-      <c r="K17" s="13"/>
-      <c r="L17" s="13"/>
-      <c r="M17" s="13"/>
-      <c r="O17" s="8"/>
-      <c r="P17" s="8"/>
-      <c r="Q17" s="8"/>
-    </row>
-    <row r="18" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="13"/>
-      <c r="J18" s="13"/>
-      <c r="K18" s="13"/>
-      <c r="L18" s="13"/>
-      <c r="M18" s="13"/>
-      <c r="O18" s="8"/>
-      <c r="P18" s="8"/>
-      <c r="Q18" s="8"/>
-    </row>
-    <row r="19" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="13"/>
-      <c r="H19" s="13"/>
-      <c r="I19" s="13"/>
-      <c r="J19" s="13"/>
-      <c r="K19" s="13"/>
-      <c r="L19" s="13"/>
-      <c r="M19" s="13"/>
-      <c r="O19" s="8"/>
-      <c r="P19" s="8"/>
-      <c r="Q19" s="8"/>
-    </row>
-    <row r="20" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="13"/>
-      <c r="H20" s="13"/>
-      <c r="I20" s="13"/>
-      <c r="J20" s="13"/>
-      <c r="K20" s="13"/>
-      <c r="L20" s="13"/>
-      <c r="M20" s="13"/>
-      <c r="O20" s="8"/>
-      <c r="P20" s="8"/>
-      <c r="Q20" s="8"/>
-    </row>
-    <row r="21" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="13"/>
-      <c r="H21" s="13"/>
-      <c r="I21" s="13"/>
-      <c r="J21" s="13"/>
-      <c r="K21" s="13"/>
-      <c r="L21" s="13"/>
-      <c r="M21" s="13"/>
-      <c r="O21" s="8"/>
-      <c r="P21" s="8"/>
-      <c r="Q21" s="8"/>
-    </row>
-    <row r="22" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="13"/>
-      <c r="H22" s="13"/>
-      <c r="I22" s="13"/>
-      <c r="J22" s="13"/>
-      <c r="K22" s="13"/>
-      <c r="L22" s="13"/>
-      <c r="M22" s="13"/>
-      <c r="O22" s="8"/>
-      <c r="P22" s="8"/>
-      <c r="Q22" s="8"/>
-    </row>
-    <row r="23" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B23" s="13"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="13"/>
-      <c r="H23" s="13"/>
-      <c r="I23" s="13"/>
-      <c r="J23" s="13"/>
-      <c r="K23" s="13"/>
-      <c r="L23" s="13"/>
-      <c r="M23" s="13"/>
-      <c r="O23" s="8"/>
-      <c r="P23" s="8"/>
-      <c r="Q23" s="8"/>
-    </row>
-    <row r="24" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="13"/>
-      <c r="H24" s="13"/>
-      <c r="I24" s="13"/>
-      <c r="J24" s="13"/>
-      <c r="K24" s="13"/>
-      <c r="L24" s="13"/>
-      <c r="M24" s="13"/>
-      <c r="O24" s="8"/>
-      <c r="P24" s="8"/>
-      <c r="Q24" s="8"/>
-    </row>
-    <row r="25" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="13"/>
-      <c r="H25" s="13"/>
-      <c r="I25" s="13"/>
-      <c r="J25" s="13"/>
-      <c r="K25" s="13"/>
-      <c r="L25" s="13"/>
-      <c r="M25" s="13"/>
-      <c r="O25" s="8"/>
-      <c r="P25" s="8"/>
-      <c r="Q25" s="8"/>
-    </row>
-    <row r="26" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="13"/>
-      <c r="G26" s="13"/>
-      <c r="H26" s="13"/>
-      <c r="I26" s="13"/>
-      <c r="J26" s="13"/>
-      <c r="K26" s="13"/>
-      <c r="L26" s="13"/>
-      <c r="M26" s="13"/>
-      <c r="O26" s="8"/>
-      <c r="P26" s="8"/>
-      <c r="Q26" s="8"/>
-    </row>
-    <row r="27" spans="15:17" x14ac:dyDescent="0.25">
-      <c r="O27" s="8"/>
-      <c r="P27" s="8"/>
-      <c r="Q27" s="8"/>
-    </row>
-    <row r="28" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B28" s="13" t="s">
-        <v>405</v>
-      </c>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
-      <c r="F28" s="13"/>
-      <c r="G28" s="13"/>
-      <c r="H28" s="13" t="s">
-        <v>406</v>
-      </c>
-      <c r="I28" s="13"/>
-      <c r="J28" s="13"/>
-      <c r="K28" s="13"/>
-      <c r="L28" s="13"/>
-      <c r="M28" s="13"/>
-      <c r="O28" s="8"/>
-      <c r="P28" s="8"/>
-      <c r="Q28" s="8"/>
-      <c r="T28" s="6" t="s">
-        <v>407</v>
-      </c>
-      <c r="U28" s="6"/>
-      <c r="V28" s="6"/>
-      <c r="W28" s="6"/>
-    </row>
-    <row r="29" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B29" s="13"/>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
-      <c r="F29" s="13"/>
-      <c r="G29" s="13"/>
-      <c r="H29" s="13"/>
-      <c r="I29" s="13"/>
-      <c r="J29" s="13"/>
-      <c r="K29" s="13"/>
-      <c r="L29" s="13"/>
-      <c r="M29" s="13"/>
-      <c r="O29" s="8"/>
-      <c r="P29" s="8"/>
-      <c r="Q29" s="8"/>
-    </row>
-    <row r="30" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B30" s="13"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="13"/>
-      <c r="G30" s="13"/>
-      <c r="H30" s="13"/>
-      <c r="I30" s="13"/>
-      <c r="J30" s="13"/>
-      <c r="K30" s="13"/>
-      <c r="L30" s="13"/>
-      <c r="M30" s="13"/>
-      <c r="O30" s="8"/>
-      <c r="P30" s="8"/>
-      <c r="Q30" s="8"/>
-    </row>
-    <row r="31" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B31" s="13"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="13"/>
-      <c r="G31" s="13"/>
-      <c r="H31" s="13"/>
-      <c r="I31" s="13"/>
-      <c r="J31" s="13"/>
-      <c r="K31" s="13"/>
-      <c r="L31" s="13"/>
-      <c r="M31" s="13"/>
-      <c r="O31" s="8"/>
-      <c r="P31" s="8"/>
-      <c r="Q31" s="8"/>
-    </row>
-    <row r="32" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B32" s="13"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="13"/>
-      <c r="H32" s="13"/>
-      <c r="I32" s="13"/>
-      <c r="J32" s="13"/>
-      <c r="K32" s="13"/>
-      <c r="L32" s="13"/>
-      <c r="M32" s="13"/>
-      <c r="O32" s="8"/>
-      <c r="P32" s="8"/>
-      <c r="Q32" s="8"/>
-    </row>
-    <row r="33" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B33" s="13"/>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
-      <c r="F33" s="13"/>
-      <c r="G33" s="13"/>
-      <c r="H33" s="13"/>
-      <c r="I33" s="13"/>
-      <c r="J33" s="13"/>
-      <c r="K33" s="13"/>
-      <c r="L33" s="13"/>
-      <c r="M33" s="13"/>
-      <c r="O33" s="8"/>
-      <c r="P33" s="8"/>
-      <c r="Q33" s="8"/>
-    </row>
-    <row r="34" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B34" s="13"/>
-      <c r="C34" s="13"/>
-      <c r="D34" s="13"/>
-      <c r="E34" s="13"/>
-      <c r="F34" s="13"/>
-      <c r="G34" s="13"/>
-      <c r="H34" s="13"/>
-      <c r="I34" s="13"/>
-      <c r="J34" s="13"/>
-      <c r="K34" s="13"/>
-      <c r="L34" s="13"/>
-      <c r="M34" s="13"/>
-      <c r="O34" s="8"/>
-      <c r="P34" s="8"/>
-      <c r="Q34" s="8"/>
-    </row>
-    <row r="35" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B35" s="13"/>
-      <c r="C35" s="13"/>
-      <c r="D35" s="13"/>
-      <c r="E35" s="13"/>
-      <c r="F35" s="13"/>
-      <c r="G35" s="13"/>
-      <c r="H35" s="13"/>
-      <c r="I35" s="13"/>
-      <c r="J35" s="13"/>
-      <c r="K35" s="13"/>
-      <c r="L35" s="13"/>
-      <c r="M35" s="13"/>
-      <c r="O35" s="8"/>
-      <c r="P35" s="8"/>
-      <c r="Q35" s="8"/>
-    </row>
-    <row r="36" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B36" s="13"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="13"/>
-      <c r="F36" s="13"/>
-      <c r="G36" s="13"/>
-      <c r="H36" s="13"/>
-      <c r="I36" s="13"/>
-      <c r="J36" s="13"/>
-      <c r="K36" s="13"/>
-      <c r="L36" s="13"/>
-      <c r="M36" s="13"/>
-      <c r="O36" s="8"/>
-      <c r="P36" s="8"/>
-      <c r="Q36" s="8"/>
-    </row>
-    <row r="37" spans="2:23" x14ac:dyDescent="0.25">
-      <c r="B37" s="13"/>
-      <c r="C37" s="13"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
-      <c r="F37" s="13"/>
-      <c r="G37" s="13"/>
-      <c r="H37" s="13"/>
-      <c r="I37" s="13"/>
-      <c r="J37" s="13"/>
-      <c r="K37" s="13"/>
-      <c r="L37" s="13"/>
-      <c r="M37" s="13"/>
-      <c r="O37" s="8"/>
-      <c r="P37" s="8"/>
-      <c r="Q37" s="8"/>
-      <c r="T37" s="6" t="s">
-        <v>408</v>
-      </c>
-      <c r="U37" s="6"/>
-      <c r="V37" s="6"/>
-      <c r="W37" s="6"/>
-    </row>
-    <row r="38" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B38" s="13"/>
-      <c r="C38" s="13"/>
-      <c r="D38" s="13"/>
-      <c r="E38" s="13"/>
-      <c r="F38" s="13"/>
-      <c r="G38" s="13"/>
-      <c r="H38" s="13"/>
-      <c r="I38" s="13"/>
-      <c r="J38" s="13"/>
-      <c r="K38" s="13"/>
-      <c r="L38" s="13"/>
-      <c r="M38" s="13"/>
-      <c r="O38" s="8"/>
-      <c r="P38" s="8"/>
-      <c r="Q38" s="8"/>
-    </row>
-    <row r="39" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B39" s="13"/>
-      <c r="C39" s="13"/>
-      <c r="D39" s="13"/>
-      <c r="E39" s="13"/>
-      <c r="F39" s="13"/>
-      <c r="G39" s="13"/>
-      <c r="H39" s="13"/>
-      <c r="I39" s="13"/>
-      <c r="J39" s="13"/>
-      <c r="K39" s="13"/>
-      <c r="L39" s="13"/>
-      <c r="M39" s="13"/>
-      <c r="O39" s="8"/>
-      <c r="P39" s="8"/>
-      <c r="Q39" s="8"/>
-    </row>
-    <row r="40" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B40" s="13"/>
-      <c r="C40" s="13"/>
-      <c r="D40" s="13"/>
-      <c r="E40" s="13"/>
-      <c r="F40" s="13"/>
-      <c r="G40" s="13"/>
-      <c r="H40" s="13"/>
-      <c r="I40" s="13"/>
-      <c r="J40" s="13"/>
-      <c r="K40" s="13"/>
-      <c r="L40" s="13"/>
-      <c r="M40" s="13"/>
-      <c r="O40" s="8"/>
-      <c r="P40" s="8"/>
-      <c r="Q40" s="8"/>
-    </row>
-    <row r="41" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B41" s="13"/>
-      <c r="C41" s="13"/>
-      <c r="D41" s="13"/>
-      <c r="E41" s="13"/>
-      <c r="F41" s="13"/>
-      <c r="G41" s="13"/>
-      <c r="H41" s="13"/>
-      <c r="I41" s="13"/>
-      <c r="J41" s="13"/>
-      <c r="K41" s="13"/>
-      <c r="L41" s="13"/>
-      <c r="M41" s="13"/>
-      <c r="O41" s="8"/>
-      <c r="P41" s="8"/>
-      <c r="Q41" s="8"/>
-    </row>
-    <row r="42" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B42" s="13"/>
-      <c r="C42" s="13"/>
-      <c r="D42" s="13"/>
-      <c r="E42" s="13"/>
-      <c r="F42" s="13"/>
-      <c r="G42" s="13"/>
-      <c r="H42" s="13"/>
-      <c r="I42" s="13"/>
-      <c r="J42" s="13"/>
-      <c r="K42" s="13"/>
-      <c r="L42" s="13"/>
-      <c r="M42" s="13"/>
-      <c r="O42" s="8"/>
-      <c r="P42" s="8"/>
-      <c r="Q42" s="8"/>
-    </row>
-    <row r="43" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B43" s="13"/>
-      <c r="C43" s="13"/>
-      <c r="D43" s="13"/>
-      <c r="E43" s="13"/>
-      <c r="F43" s="13"/>
-      <c r="G43" s="13"/>
-      <c r="H43" s="13"/>
-      <c r="I43" s="13"/>
-      <c r="J43" s="13"/>
-      <c r="K43" s="13"/>
-      <c r="L43" s="13"/>
-      <c r="M43" s="13"/>
-      <c r="O43" s="8"/>
-      <c r="P43" s="8"/>
-      <c r="Q43" s="8"/>
-    </row>
-    <row r="45" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B45" s="14" t="s">
-        <v>409</v>
-      </c>
-      <c r="C45" s="14"/>
-      <c r="D45" s="14"/>
-      <c r="E45" s="14"/>
-      <c r="F45" s="14"/>
-      <c r="G45" s="14"/>
-      <c r="H45" s="14"/>
-      <c r="I45" s="14"/>
-      <c r="J45" s="14"/>
-      <c r="K45" s="14"/>
-      <c r="L45" s="14"/>
-      <c r="M45" s="14"/>
-      <c r="N45" s="14"/>
-      <c r="O45" s="14"/>
-      <c r="P45" s="14"/>
-      <c r="Q45" s="14"/>
-    </row>
-    <row r="46" ht="30" customHeight="1" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B46" s="15" t="s">
-        <v>410</v>
-      </c>
-      <c r="C46" s="15"/>
-      <c r="D46" s="15"/>
-      <c r="E46" s="15"/>
-      <c r="F46" s="15"/>
-      <c r="G46" s="15"/>
-      <c r="H46" s="15"/>
-      <c r="I46" s="15"/>
-      <c r="J46" s="15"/>
-      <c r="K46" s="15"/>
-      <c r="L46" s="15"/>
-      <c r="M46" s="15"/>
-      <c r="N46" s="15"/>
-      <c r="O46" s="15"/>
-      <c r="P46" s="15"/>
-      <c r="Q46" s="15"/>
-    </row>
-    <row r="47" ht="30" customHeight="1" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B47" s="15" t="s">
-        <v>411</v>
-      </c>
-      <c r="C47" s="15"/>
-      <c r="D47" s="15"/>
-      <c r="E47" s="15"/>
-      <c r="F47" s="15"/>
-      <c r="G47" s="15"/>
-      <c r="H47" s="15"/>
-      <c r="I47" s="15"/>
-      <c r="J47" s="15"/>
-      <c r="K47" s="15"/>
-      <c r="L47" s="15"/>
-      <c r="M47" s="15"/>
-      <c r="N47" s="15"/>
-      <c r="O47" s="15"/>
-      <c r="P47" s="15"/>
-      <c r="Q47" s="15"/>
-    </row>
-    <row r="48" ht="30" customHeight="1" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B48" s="15" t="s">
-        <v>412</v>
-      </c>
-      <c r="C48" s="15"/>
-      <c r="D48" s="15"/>
-      <c r="E48" s="15"/>
-      <c r="F48" s="15"/>
-      <c r="G48" s="15"/>
-      <c r="H48" s="15"/>
-      <c r="I48" s="15"/>
-      <c r="J48" s="15"/>
-      <c r="K48" s="15"/>
-      <c r="L48" s="15"/>
-      <c r="M48" s="15"/>
-      <c r="N48" s="15"/>
-      <c r="O48" s="15"/>
-      <c r="P48" s="15"/>
-      <c r="Q48" s="15"/>
-    </row>
-  </sheetData>
-  <mergeCells count="22">
-    <mergeCell ref="B1:Q2"/>
-    <mergeCell ref="B3:Q3"/>
-    <mergeCell ref="T3:W3"/>
-    <mergeCell ref="T4:W4"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="F5:I5"/>
-    <mergeCell ref="J5:M5"/>
-    <mergeCell ref="O5:Q43"/>
-    <mergeCell ref="B6:E8"/>
-    <mergeCell ref="F6:I8"/>
-    <mergeCell ref="J6:M8"/>
-    <mergeCell ref="B9:M9"/>
-    <mergeCell ref="T9:W9"/>
-    <mergeCell ref="B11:M26"/>
-    <mergeCell ref="B28:G43"/>
-    <mergeCell ref="H28:M43"/>
-    <mergeCell ref="T28:W28"/>
-    <mergeCell ref="T37:W37"/>
-    <mergeCell ref="B45:Q45"/>
-    <mergeCell ref="B46:Q46"/>
-    <mergeCell ref="B47:Q47"/>
-    <mergeCell ref="B48:Q48"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Módulo 4: montos en formato de moneda RD$ (tablas, ejes y base Excel) y punto final en los títulos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Modulo4-Base-Dashboard.xlsx
+++ b/Modulo4-Base-Dashboard.xlsx
@@ -1196,8 +1196,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="&quot;RD$&quot; #,##0.00"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -1231,7 +1232,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1608,7 +1609,7 @@
     <col min="4" max="4" width="29" customWidth="1"/>
     <col min="5" max="5" width="17" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="13" style="2" customWidth="1"/>
+    <col min="7" max="7" width="16" style="2" customWidth="1"/>
     <col min="8" max="8" width="8" customWidth="1"/>
     <col min="9" max="9" width="7" customWidth="1"/>
   </cols>

</xml_diff>